<commit_message>
🎨 Harmonisation pastel des 3 feuilles + Saisie reformulée comme tableau panel
</commit_message>
<xml_diff>
--- a/tableau-de-bord-pro/tableau-de-bord-pro.xlsx
+++ b/tableau-de-bord-pro/tableau-de-bord-pro.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,8 +63,27 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <color rgb="002C3A47"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005B7C8D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002C3A47"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -106,8 +125,32 @@
         <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B7C8D"/>
+        <bgColor rgb="005B7C8D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF4F8"/>
+        <bgColor rgb="00EFF4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008FAEC0"/>
+        <bgColor rgb="008FAEC0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+        <bgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -149,11 +192,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBCCDA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BBCCDA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBCCDA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBCCDA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -186,11 +243,38 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -202,6 +286,22 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFE4E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E5F0DD"/>
+          <bgColor rgb="00E5F0DD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F5DDDE"/>
+          <bgColor rgb="00F5DDDE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -585,114 +685,117 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Prénom</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Âge</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>Date d'ajout</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>Dernière MAJ</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>DUPONT</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>Martin</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="17" t="n">
         <v>42</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="18" t="n">
         <v>46281</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>Actif</t>
         </is>
       </c>
+      <c r="F2" s="17" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>MARTIN</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Sophie</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="17" t="n">
         <v>29</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="18" t="n">
         <v>46281</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>Périmé</t>
         </is>
       </c>
+      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>BENALI</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Karim</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="17" t="n">
         <v>35</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="18" t="n">
         <v>46281</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Actif</t>
         </is>
       </c>
+      <c r="F4" s="17" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F50"/>
@@ -701,6 +804,14 @@
       <formula>"Actif"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Périmé"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F4">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Actif"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Périmé"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -722,81 +833,75 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>📋 SAISIE D'UN NOUVEAU DOSSIER</t>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>📋 Saisie d'un nouveau dossier</t>
         </is>
       </c>
       <c r="B1" s="4" t="n"/>
       <c r="C1" s="5" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Nom de famille</t>
-        </is>
-      </c>
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Prénom</t>
         </is>
       </c>
+      <c r="B5" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Âge</t>
         </is>
       </c>
+      <c r="B7" s="21" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
+      <c r="B9" s="21" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Date d'ajout</t>
-        </is>
-      </c>
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Date ajout</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Dernière MAJ</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ Cliquez sur le bouton ➡️</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B13" s="21" t="n"/>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>🟢 ENREGISTRER DANS DOSSIERS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>La ligne est ajoutée en bas de la feuille Dossiers (préservée même en tablet Google etc.)</t>
         </is>
       </c>
     </row>
@@ -830,27 +935,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>🟢 Actif</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="23" t="inlineStr">
         <is>
           <t>🖍 En cours</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="23" t="inlineStr">
         <is>
           <t>🔴 Périmé</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>✔️ Fermé</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="23" t="inlineStr">
         <is>
           <t>➕ Autre</t>
         </is>

</xml_diff>